<commit_message>
feat: remove adaptatutexto and update groups
</commit_message>
<xml_diff>
--- a/notebooks/01_first_analysis/analisis_herramientas_completo.xlsx
+++ b/notebooks/01_first_analysis/analisis_herramientas_completo.xlsx
@@ -1659,7 +1659,7 @@
       </c>
       <c r="EK2" t="inlineStr">
         <is>
-          <t>Modelos IA</t>
+          <t>Grupo 1: Agentes Conversacionales</t>
         </is>
       </c>
       <c r="EL2" t="n">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="EK3" t="inlineStr">
         <is>
-          <t>Modelos IA</t>
+          <t>Grupo 1: Agentes Conversacionales</t>
         </is>
       </c>
       <c r="EL3" t="n">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="EK4" t="inlineStr">
         <is>
-          <t>Modelos IA</t>
+          <t>Grupo 1: Agentes Conversacionales</t>
         </is>
       </c>
       <c r="EL4" t="n">
@@ -3255,7 +3255,7 @@
       </c>
       <c r="EK5" t="inlineStr">
         <is>
-          <t>Modelos IA</t>
+          <t>Grupo 1: Agentes Conversacionales</t>
         </is>
       </c>
       <c r="EL5" t="n">
@@ -3787,7 +3787,7 @@
       </c>
       <c r="EK6" t="inlineStr">
         <is>
-          <t>Modelos IA</t>
+          <t>Grupo 1: Agentes Conversacionales</t>
         </is>
       </c>
       <c r="EL6" t="n">
@@ -4319,7 +4319,7 @@
       </c>
       <c r="EK7" t="inlineStr">
         <is>
-          <t>Modelos IA</t>
+          <t>Grupo 1: Agentes Conversacionales</t>
         </is>
       </c>
       <c r="EL7" t="n">
@@ -4851,7 +4851,7 @@
       </c>
       <c r="EK8" t="inlineStr">
         <is>
-          <t>Modelos IA</t>
+          <t>Grupo 1: Agentes Conversacionales</t>
         </is>
       </c>
       <c r="EL8" t="n">
@@ -5380,11 +5380,7 @@
       <c r="EJ9" t="n">
         <v>19</v>
       </c>
-      <c r="EK9" t="inlineStr">
-        <is>
-          <t>Modelos IA</t>
-        </is>
-      </c>
+      <c r="EK9" t="inlineStr"/>
       <c r="EL9" t="n">
         <v>13.5</v>
       </c>
@@ -5911,11 +5907,7 @@
       <c r="EJ10" t="n">
         <v>18</v>
       </c>
-      <c r="EK10" t="inlineStr">
-        <is>
-          <t>Modelos IA</t>
-        </is>
-      </c>
+      <c r="EK10" t="inlineStr"/>
       <c r="EL10" t="n">
         <v>14.5</v>
       </c>
@@ -6442,11 +6434,7 @@
       <c r="EJ11" t="n">
         <v>17</v>
       </c>
-      <c r="EK11" t="inlineStr">
-        <is>
-          <t>Modelos IA</t>
-        </is>
-      </c>
+      <c r="EK11" t="inlineStr"/>
       <c r="EL11" t="n">
         <v>13.5</v>
       </c>
@@ -6975,7 +6963,7 @@
       </c>
       <c r="EK12" t="inlineStr">
         <is>
-          <t>Modelos IA</t>
+          <t>Grupo 2: Modelos Fundacionales</t>
         </is>
       </c>
       <c r="EL12" t="n">
@@ -7506,7 +7494,7 @@
       </c>
       <c r="EK13" t="inlineStr">
         <is>
-          <t>Normas UNE</t>
+          <t>Grupo 3: Norma UNE</t>
         </is>
       </c>
       <c r="EL13" t="n">
@@ -8037,7 +8025,7 @@
       </c>
       <c r="EK14" t="inlineStr">
         <is>
-          <t>Modelos IA</t>
+          <t>Grupo 2: Modelos Fundacionales</t>
         </is>
       </c>
       <c r="EL14" t="n">
@@ -8568,7 +8556,7 @@
       </c>
       <c r="EK15" t="inlineStr">
         <is>
-          <t>Modelos IA</t>
+          <t>Grupo 2: Modelos Fundacionales</t>
         </is>
       </c>
       <c r="EL15" t="n">
@@ -9099,7 +9087,7 @@
       </c>
       <c r="EK16" t="inlineStr">
         <is>
-          <t>Modelos IA</t>
+          <t>Grupo 3: Norma UNE</t>
         </is>
       </c>
       <c r="EL16" t="n">
@@ -9628,11 +9616,7 @@
       <c r="EJ17" t="n">
         <v>20</v>
       </c>
-      <c r="EK17" t="inlineStr">
-        <is>
-          <t>Modelos IA</t>
-        </is>
-      </c>
+      <c r="EK17" t="inlineStr"/>
       <c r="EL17" t="n">
         <v>13.5</v>
       </c>
@@ -10161,7 +10145,7 @@
       </c>
       <c r="EK18" t="inlineStr">
         <is>
-          <t>Normas UNE</t>
+          <t>Grupo 3: Norma UNE</t>
         </is>
       </c>
       <c r="EL18" t="n">
@@ -10692,7 +10676,7 @@
       </c>
       <c r="EK19" t="inlineStr">
         <is>
-          <t>Modelos IA</t>
+          <t>Grupo 2: Modelos Fundacionales</t>
         </is>
       </c>
       <c r="EL19" t="n">

</xml_diff>

<commit_message>
feat: update data and metrics
</commit_message>
<xml_diff>
--- a/notebooks/01_first_analysis/analisis_herramientas_completo.xlsx
+++ b/notebooks/01_first_analysis/analisis_herramientas_completo.xlsx
@@ -1662,16 +1662,16 @@
         </is>
       </c>
       <c r="EL2" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="EM2" t="n">
-        <v>100</v>
+        <v>86.667</v>
       </c>
       <c r="EN2" t="n">
-        <v>0.3185577778255009</v>
+        <v>0.2842303091606552</v>
       </c>
       <c r="EO2" t="n">
-        <v>0.6720324441540493</v>
+        <v>0.6515941062416063</v>
       </c>
     </row>
     <row r="3">
@@ -2193,16 +2193,16 @@
         </is>
       </c>
       <c r="EL3" t="n">
-        <v>14.5</v>
+        <v>14</v>
       </c>
       <c r="EM3" t="n">
-        <v>96.667</v>
+        <v>93.333</v>
       </c>
       <c r="EN3" t="n">
-        <v>0.3856158540135085</v>
+        <v>0.3847019839046188</v>
       </c>
       <c r="EO3" t="n">
-        <v>0.4861239730659023</v>
+        <v>0.5152437366123078</v>
       </c>
     </row>
     <row r="4">
@@ -2724,16 +2724,16 @@
         </is>
       </c>
       <c r="EL4" t="n">
-        <v>13.5</v>
+        <v>12</v>
       </c>
       <c r="EM4" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="EN4" t="n">
-        <v>0.3447398172411324</v>
+        <v>0.3560382939968362</v>
       </c>
       <c r="EO4" t="n">
-        <v>0.536325126515934</v>
+        <v>0.5671133252470847</v>
       </c>
     </row>
     <row r="5">
@@ -3255,16 +3255,16 @@
         </is>
       </c>
       <c r="EL5" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="EM5" t="n">
-        <v>73.333</v>
+        <v>93.333</v>
       </c>
       <c r="EN5" t="n">
-        <v>0.3079803388692983</v>
+        <v>0.3100958423921303</v>
       </c>
       <c r="EO5" t="n">
-        <v>0.3960929989749037</v>
+        <v>0.4971079350151025</v>
       </c>
     </row>
     <row r="6">
@@ -3792,10 +3792,10 @@
         <v>93.333</v>
       </c>
       <c r="EN6" t="n">
-        <v>0.4367833884739029</v>
+        <v>0.455462139248744</v>
       </c>
       <c r="EO6" t="n">
-        <v>0.5212817704440919</v>
+        <v>0.5050707157986412</v>
       </c>
     </row>
     <row r="7">
@@ -4317,16 +4317,16 @@
         </is>
       </c>
       <c r="EL7" t="n">
-        <v>12.5</v>
+        <v>14</v>
       </c>
       <c r="EM7" t="n">
-        <v>83.333</v>
+        <v>93.333</v>
       </c>
       <c r="EN7" t="n">
-        <v>0.2779923184022218</v>
+        <v>0.2697181161238288</v>
       </c>
       <c r="EO7" t="n">
-        <v>0.7001293829780103</v>
+        <v>0.7345368369700467</v>
       </c>
     </row>
     <row r="8">
@@ -4848,16 +4848,16 @@
         </is>
       </c>
       <c r="EL8" t="n">
-        <v>11.5</v>
+        <v>12</v>
       </c>
       <c r="EM8" t="n">
-        <v>76.667</v>
+        <v>80</v>
       </c>
       <c r="EN8" t="n">
-        <v>0.3821666255109876</v>
+        <v>0.3673872877332308</v>
       </c>
       <c r="EO8" t="n">
-        <v>0.4553311873517535</v>
+        <v>0.5305407749762505</v>
       </c>
     </row>
     <row r="9">
@@ -5379,16 +5379,16 @@
         </is>
       </c>
       <c r="EL9" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="EM9" t="n">
-        <v>93.333</v>
+        <v>66.667</v>
       </c>
       <c r="EN9" t="n">
-        <v>0.3178395777650641</v>
+        <v>0.3350956677929117</v>
       </c>
       <c r="EO9" t="n">
-        <v>0.5088267764091003</v>
+        <v>0.4589088546391809</v>
       </c>
     </row>
     <row r="10">
@@ -5910,16 +5910,16 @@
         </is>
       </c>
       <c r="EL10" t="n">
-        <v>13.5</v>
+        <v>12</v>
       </c>
       <c r="EM10" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="EN10" t="n">
-        <v>0.3396612465022376</v>
+        <v>0.3478590791260158</v>
       </c>
       <c r="EO10" t="n">
-        <v>0.4705210862541721</v>
+        <v>0.5002634567949098</v>
       </c>
     </row>
     <row r="11">
@@ -6441,16 +6441,16 @@
         </is>
       </c>
       <c r="EL11" t="n">
-        <v>12.5</v>
+        <v>14</v>
       </c>
       <c r="EM11" t="n">
-        <v>83.333</v>
+        <v>93.333</v>
       </c>
       <c r="EN11" t="n">
-        <v>0.3700561378057017</v>
+        <v>0.4125633224440607</v>
       </c>
       <c r="EO11" t="n">
-        <v>0.5941870518400698</v>
+        <v>0.5969886550765551</v>
       </c>
     </row>
     <row r="12">
@@ -6972,16 +6972,16 @@
         </is>
       </c>
       <c r="EL12" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="EM12" t="n">
-        <v>80</v>
+        <v>93.333</v>
       </c>
       <c r="EN12" t="n">
-        <v>0.368827885993098</v>
+        <v>0.3339621580072221</v>
       </c>
       <c r="EO12" t="n">
-        <v>0.6715706900218524</v>
+        <v>0.7590371168313065</v>
       </c>
     </row>
   </sheetData>

</xml_diff>